<commit_message>
refactor: improve rounding logic for financial calculations and update number formatting in SummaryPreview
</commit_message>
<xml_diff>
--- a/backend/src/template/RCM_Payment_Template.xlsx
+++ b/backend/src/template/RCM_Payment_Template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hp\Desktop\own_pr\Kr\kr_ferm\backend\src\template\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B14DD581-3E3A-4ADC-B2ED-84D2AB7D3F6C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A3EF78E2-B278-4F8B-95C9-859F191E7573}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{1CCA70F8-4381-4395-B00F-273B2849737A}"/>
   </bookViews>
@@ -117,7 +117,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -140,28 +140,12 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -171,14 +155,17 @@
     <xf numFmtId="4" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="4" fontId="3" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -509,67 +496,67 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
-      <c r="G1" s="1"/>
-      <c r="H1" s="1"/>
-      <c r="I1" s="1"/>
-      <c r="J1" s="1"/>
-      <c r="K1" s="1"/>
+      <c r="B1" s="4"/>
+      <c r="C1" s="4"/>
+      <c r="D1" s="4"/>
+      <c r="E1" s="4"/>
+      <c r="F1" s="4"/>
+      <c r="G1" s="4"/>
+      <c r="H1" s="4"/>
+      <c r="I1" s="4"/>
+      <c r="J1" s="4"/>
+      <c r="K1" s="4"/>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A2" s="1" t="s">
+      <c r="A2" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="1"/>
-      <c r="C2" s="1"/>
-      <c r="D2" s="1"/>
-      <c r="E2" s="1"/>
-      <c r="F2" s="1"/>
-      <c r="G2" s="1"/>
-      <c r="H2" s="1"/>
-      <c r="I2" s="1"/>
-      <c r="J2" s="1"/>
-      <c r="K2" s="1"/>
+      <c r="B2" s="4"/>
+      <c r="C2" s="4"/>
+      <c r="D2" s="4"/>
+      <c r="E2" s="4"/>
+      <c r="F2" s="4"/>
+      <c r="G2" s="4"/>
+      <c r="H2" s="4"/>
+      <c r="I2" s="4"/>
+      <c r="J2" s="4"/>
+      <c r="K2" s="4"/>
     </row>
     <row r="3" spans="1:11" ht="20.399999999999999" x14ac:dyDescent="0.3">
-      <c r="A3" s="2" t="s">
+      <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="C3" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="D3" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="E3" s="2" t="s">
+      <c r="E3" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="F3" s="2" t="s">
+      <c r="F3" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="G3" s="2" t="s">
+      <c r="G3" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="H3" s="2" t="s">
+      <c r="H3" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="I3" s="2" t="s">
+      <c r="I3" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="J3" s="2" t="s">
+      <c r="J3" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="K3" s="2" t="s">
+      <c r="K3" s="1" t="s">
         <v>6</v>
       </c>
     </row>
@@ -577,38 +564,38 @@
       <c r="A4" s="5">
         <v>3</v>
       </c>
-      <c r="B4" s="7" t="s">
+      <c r="B4" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="C4" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="D4" s="4">
+      <c r="D4" s="3">
         <v>111946</v>
       </c>
-      <c r="E4" s="6">
+      <c r="E4" s="7">
         <f>+SUM(D4:D4)</f>
         <v>111946</v>
       </c>
-      <c r="F4" s="4">
+      <c r="F4" s="3">
         <v>0</v>
       </c>
-      <c r="G4" s="6">
+      <c r="G4" s="7">
         <f>+SUM(F4:F4)</f>
         <v>0</v>
       </c>
-      <c r="H4" s="6">
+      <c r="H4" s="7">
         <f>+E4-G4</f>
         <v>111946</v>
       </c>
-      <c r="I4" s="6">
+      <c r="I4" s="7">
         <f>+ROUND(E4*1%,0)</f>
         <v>1119</v>
       </c>
-      <c r="J4" s="6">
+      <c r="J4" s="7">
         <v>0</v>
       </c>
-      <c r="K4" s="6">
+      <c r="K4" s="7">
         <f>+H4-I4-J4</f>
         <v>110827</v>
       </c>

</xml_diff>